<commit_message>
Stage 8 fixes: D-009
</commit_message>
<xml_diff>
--- a/output/archive/QuenverellData/engagements/qv.23.100/rnaseq/processed/corvenlith-donor-adjusted-targets-v4.xlsx
+++ b/output/archive/QuenverellData/engagements/qv.23.100/rnaseq/processed/corvenlith-donor-adjusted-targets-v4.xlsx
@@ -170,7 +170,7 @@
   <commentList>
     <comment ref="E2" authorId="0" shapeId="0">
       <text>
-        <t>Keep the first-pass row so the change from the adjustment can be traced</t>
+        <t>Qualitative context only; obtain identified contrast output before citing effect sizes or probabilities.</t>
       </text>
     </comment>
   </commentList>
@@ -185,7 +185,7 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Ranking is donor-balanced; the earlier order is in the first-pass sheet</t>
+        <t>Decision summary only. Identify the pathway accession and analysis-output version before treating this as a reproducible ranking.</t>
       </text>
     </comment>
   </commentList>
@@ -641,102 +641,102 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cell population</t>
+          <t>Biological question</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Immune cells, bulk RNA-seq, one library per donor per condition</t>
+          <t>Immune-cell RNA-seq; donor-balanced target prioritisation</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Donor is the unit of replication</t>
+          <t>Donor is the biological replication unit.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Donor balance</t>
+          <t>Donor balance assumption</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Each condition represented by the same donors; donors with a missing condition excluded from the paired model</t>
+          <t>Sample manifest under QDATA2023-0617</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Balance check run before any contrast was fitted</t>
+          <t>Paired analysis assumes matched donors across conditions. Missing-condition/exclusion handling must be read from manifest and analysis specification; not asserted here.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Donor covariate</t>
+          <t>Model and fitting</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Donor entered as a random term; sex and collection batch as fixed covariates</t>
+          <t>Engagement analysis specification and executed analysis output under QDATA2023-0617</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Batch confirmed against the sample sheet</t>
+          <t>Condition coefficient, formula, donor structure and mixed-model fitting method are not transcribed. Do not infer a random term or fitted covariates from this summary.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Normalisation</t>
+          <t>Normalisation / filtering</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Library-size normalised counts, filtered to genes expressed in at least a quarter of samples per group</t>
+          <t>Same analysis specification and executed preprocessing record</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Filter threshold set before fitting</t>
+          <t>Normalisation algorithm and filtering parameters not reproduced.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Significance</t>
+          <t>Multiplicity</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Adjusted probability threshold 0.05 across all contrasts</t>
+          <t>Specification and contrast-output metadata</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Thresholds fixed in the analysis plan</t>
+          <t>Correction method and tested family of genes/contrasts must be identified there; no universal 0.05 acceptance claim.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Effect size</t>
+          <t>Reproducibility limit</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Log2 fold change reported with the adjusted probability for every contrast</t>
+          <t>Exact specification/output filenames and versions are not identified in this summary</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Fold changes on the log2 scale only</t>
+          <t>Retrieve the engagement analysis record before reproducing or citing a numerical result.</t>
         </is>
       </c>
     </row>
@@ -756,7 +756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -769,135 +769,67 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Contrast</t>
+          <t>Comparison context</t>
         </is>
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
-          <t>Comparison</t>
+          <t>Qualitative interpretation</t>
         </is>
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
-          <t>Log2 fold change</t>
+          <t>Source</t>
         </is>
       </c>
       <c r="D1" s="4" t="inlineStr">
         <is>
-          <t>Adjusted probability</t>
-        </is>
-      </c>
-      <c r="E1" s="4" t="inlineStr">
-        <is>
-          <t>Status</t>
+          <t>Numerical scope</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Unadjusted, all donors</t>
+          <t>Before donor balancing</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Stimulated versus resting</t>
+          <t>Apparent inflammatory signature</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>First pass, before adjustment</t>
+          <t>D-004: corvenlith-pathway-readout_v3_FINAL_final.pptx, engagement readouts directory</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Before donor adjustment</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Superseded: retained as context</t>
-        </is>
-      </c>
+          <t>Earlier interpretation retained as context; no numerical contrast reproduced.</t>
+        </is>
+      </c>
+      <c r="E2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Donor-adjusted</t>
+          <t>After donor balancing</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Stimulated versus resting, donor as random term</t>
+          <t>Apparent inflammatory signature reduced</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Reported in readout v3</t>
+          <t>Same D-004 readout; analysis records under QDATA2023-0617</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Adjusted, threshold 0.05</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Final</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Receptor pathway</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Pathway-level contrast, donor-adjusted</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Reported in readout v3</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Adjusted, threshold 0.05</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Final</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Inflammatory signature</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Signature score, unadjusted and adjusted</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Smaller after adjustment</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Reduced after adjustment</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Final: smaller than first pass</t>
+          <t>Exact condition coefficients, log2 fold changes and adjusted probabilities not transcribed.</t>
         </is>
       </c>
     </row>
@@ -914,7 +846,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -926,88 +858,66 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Rank order</t>
+          <t>Decision theme</t>
         </is>
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
-          <t>Pathway</t>
+          <t>Recorded direction</t>
         </is>
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
-          <t>Basis</t>
+          <t>Source</t>
         </is>
       </c>
       <c r="D1" s="4" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>Identifier / ranking scope</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>First</t>
+          <t>Reproducible receptor pathway</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Receptor pathway</t>
+          <t>Prioritised for target work after donor balancing</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Holds across donors after adjustment</t>
+          <t>D-004: corvenlith-pathway-readout_v3_FINAL_final.pptx</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Prioritised for target work</t>
+          <t>Pathway database identifier and exact ranking output not recorded here; not a numbered target ranking.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Second</t>
+          <t>Apparent inflammatory signature</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Inflammatory signature</t>
+          <t>Reduced after donor balancing</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Driven by a subset of donors before adjustment</t>
+          <t>Same D-004 readout</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Deprioritised as the lead signal</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Third</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Other pathways</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Inconsistent across donors</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Not progressed</t>
+          <t>Signature definition and numerical evidence remain in engagement analysis records under QDATA2023-0617.</t>
         </is>
       </c>
     </row>

</xml_diff>